<commit_message>
Backend testing report updated
</commit_message>
<xml_diff>
--- a/testing/docs/backend/NeuChess_TesztJegyzokonyv_backend.xlsx
+++ b/testing/docs/backend/NeuChess_TesztJegyzokonyv_backend.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Oláh Ádám\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34290B34-2BE6-4CB3-8D9D-8D97E8907B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40721AC3-3F8A-4582-9DBE-950E66AFC27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="338">
   <si>
     <t>Teszt azonosító</t>
   </si>
@@ -369,51 +369,150 @@
     <t>TC-037</t>
   </si>
   <si>
+    <t>testValidMessagePasses</t>
+  </si>
+  <si>
+    <t>Érvényes üzenet – nincs hiba: 'Hello, good game!'</t>
+  </si>
+  <si>
+    <t>0,018 s</t>
+  </si>
+  <si>
     <t>TC-038</t>
   </si>
   <si>
+    <t>testSingleCharacterPasses</t>
+  </si>
+  <si>
+    <t>Egy betűs üzenet érvényes: 'a'</t>
+  </si>
+  <si>
     <t>TC-039</t>
   </si>
   <si>
+    <t>testNonStringFails</t>
+  </si>
+  <si>
+    <t>Nem string érték → hibát dob (42)</t>
+  </si>
+  <si>
     <t>TC-040</t>
   </si>
   <si>
+    <t>testEmptyStringFails</t>
+  </si>
+  <si>
+    <t>Üres string → hibát dob</t>
+  </si>
+  <si>
     <t>TC-041</t>
   </si>
   <si>
+    <t>testWhitespaceOnlyFails</t>
+  </si>
+  <si>
+    <t>Csak szóközök → hibát dob (trim után üres)</t>
+  </si>
+  <si>
     <t>TC-042</t>
   </si>
   <si>
+    <t>test101CharactersFails</t>
+  </si>
+  <si>
+    <t>101 karakter → hibát dob (határérték)</t>
+  </si>
+  <si>
     <t>TC-043</t>
   </si>
   <si>
+    <t>testEnglishBannedWordFails</t>
+  </si>
+  <si>
+    <t>Angol tiltott szó 'fuck' → inappropriate hiba</t>
+  </si>
+  <si>
     <t>TC-044</t>
   </si>
   <si>
+    <t>testHungarianBannedWordFails</t>
+  </si>
+  <si>
+    <t>Magyar tiltott szó 'kurva' → inappropriate hiba</t>
+  </si>
+  <si>
     <t>TC-045</t>
   </si>
   <si>
+    <t>testLeetSpeakBannedWordFails</t>
+  </si>
+  <si>
+    <t>Leetspeak tiltott szó 'f4ggot' → hiba</t>
+  </si>
+  <si>
     <t>TC-046</t>
   </si>
   <si>
+    <t>testPatternBasedBannedWordFails</t>
+  </si>
+  <si>
+    <t>Regex-minta 'f*ck' → inappropriate hiba</t>
+  </si>
+  <si>
     <t>TC-047</t>
   </si>
   <si>
+    <t>testExcessiveCapitalizationFails</t>
+  </si>
+  <si>
+    <t>Túlzott nagybetűsítés &gt;70% → capitalization hiba</t>
+  </si>
+  <si>
     <t>TC-048</t>
   </si>
   <si>
+    <t>testNormalCapitalizationPasses</t>
+  </si>
+  <si>
+    <t>Normális nagybetűsítés → nincs hiba</t>
+  </si>
+  <si>
     <t>TC-049</t>
   </si>
   <si>
+    <t>testRepeatedCharactersFail</t>
+  </si>
+  <si>
+    <t>7+ ismétlődő karakter → repeated hiba</t>
+  </si>
+  <si>
     <t>TC-050</t>
   </si>
   <si>
+    <t>testSixRepeatedCharactersPasses</t>
+  </si>
+  <si>
+    <t>6 ismétlődő karakter (határérték) → nincs hiba</t>
+  </si>
+  <si>
     <t>TC-051</t>
   </si>
   <si>
+    <t>testNoLettersFails</t>
+  </si>
+  <si>
+    <t>Csak számok/szimbólumok betű nélkül → readable hiba</t>
+  </si>
+  <si>
     <t>TC-052</t>
   </si>
   <si>
+    <t>testMessageWithNumbersAndLetterPasses</t>
+  </si>
+  <si>
+    <t>Szám + legalább egy betű → érvényes</t>
+  </si>
+  <si>
     <t>TC-053</t>
   </si>
   <si>
@@ -465,9 +564,21 @@
     <t>TC-058</t>
   </si>
   <si>
+    <t>testValidBase64ButNotImageFails</t>
+  </si>
+  <si>
+    <t>Érvényes base64, de nem kép tartalom → hiba</t>
+  </si>
+  <si>
     <t>TC-059</t>
   </si>
   <si>
+    <t>testJpegPrefixIsAcceptedFormat</t>
+  </si>
+  <si>
+    <t>JPEG prefix elfogadott – JPEG or PNG hiba nem jelenik meg</t>
+  </si>
+  <si>
     <t>TC-060</t>
   </si>
   <si>
@@ -648,42 +759,147 @@
     <t>0,042 s</t>
   </si>
   <si>
+    <t>TC-079</t>
+  </si>
+  <si>
     <t>testCreateDataStoreRemovesSpacesFromDurationInMatchId</t>
   </si>
   <si>
     <t>createDataStore – Szóközök eltávolítása duration-ből: '10|0-room'</t>
   </si>
   <si>
+    <t>TC-080</t>
+  </si>
+  <si>
     <t>testCreateDataStorePlayedAtIsRecent</t>
   </si>
   <si>
     <t>createDataStore – PlayedAt aktuális időpont</t>
   </si>
   <si>
+    <t>TC-081</t>
+  </si>
+  <si>
     <t>testCreateDataStoreInitializesEmptyChatMessages</t>
   </si>
   <si>
     <t>createDataStore – Üres ChatMessages inicializálás</t>
   </si>
   <si>
+    <t>TC-082</t>
+  </si>
+  <si>
     <t>testCreateDataStoreSetsMatchDurationOnMatchState</t>
   </si>
   <si>
     <t>createDataStore – MatchDuration beállítva MatchState-en</t>
   </si>
   <si>
+    <t>TC-083</t>
+  </si>
+  <si>
     <t>testCreateDataStoreCreatesTwoPlayers</t>
   </si>
   <si>
     <t>createDataStore – Két játékos létrehozva, ID-k helyesek</t>
   </si>
   <si>
+    <t>TC-084</t>
+  </si>
+  <si>
     <t>testCreateDataStoreClocksMatchDuration</t>
   </si>
   <si>
     <t>createDataStore – Óra alap ms: WhiteRemainingMs=180000</t>
   </si>
   <si>
+    <t>TC-085</t>
+  </si>
+  <si>
+    <t>testValidMessageReturnsSuccessStatus</t>
+  </si>
+  <si>
+    <t>Érvényes üzenet → Status='Success'</t>
+  </si>
+  <si>
+    <t>0,019 s</t>
+  </si>
+  <si>
+    <t>TC-086</t>
+  </si>
+  <si>
+    <t>testValidMessageReturnsNewMessageData</t>
+  </si>
+  <si>
+    <t>Érvényes üzenet → NewMessage tartalmazza a UserID-t és üzenetet</t>
+  </si>
+  <si>
+    <t>TC-087</t>
+  </si>
+  <si>
+    <t>testValidMessageIsAppendedToChatMessages</t>
+  </si>
+  <si>
+    <t>Két érvényes üzenet felhalmozódik (count=2, sorrend helyes)</t>
+  </si>
+  <si>
+    <t>TC-088</t>
+  </si>
+  <si>
+    <t>testValidMessageStoresCorrectUserId</t>
+  </si>
+  <si>
+    <t>Helyes UserID tárolása a ChatMessages-ben</t>
+  </si>
+  <si>
+    <t>TC-089</t>
+  </si>
+  <si>
+    <t>testSingleCharacterMessageIsValid</t>
+  </si>
+  <si>
+    <t>1 karakteres üzenet érvényes → Success</t>
+  </si>
+  <si>
+    <t>TC-090</t>
+  </si>
+  <si>
+    <t>testMessageExceeding100CharsReturnsViolation</t>
+  </si>
+  <si>
+    <t>101 karakteres üzenet → Status='Violation'</t>
+  </si>
+  <si>
+    <t>TC-091</t>
+  </si>
+  <si>
+    <t>testBannedEnglishWordReturnsViolation</t>
+  </si>
+  <si>
+    <t>Tiltott angol szó → Status='Violation'</t>
+  </si>
+  <si>
+    <t>TC-092</t>
+  </si>
+  <si>
+    <t>testBannedHungarianWordReturnsViolation</t>
+  </si>
+  <si>
+    <t>Tiltott magyar szó → Status='Violation'</t>
+  </si>
+  <si>
+    <t>TC-093</t>
+  </si>
+  <si>
+    <t>testMultipleValidMessagesAccumulate</t>
+  </si>
+  <si>
+    <t>5 érvényes üzenet sorban → count=5</t>
+  </si>
+  <si>
+    <t>TC-094</t>
+  </si>
+  <si>
     <t>testPawnSimpleMove</t>
   </si>
   <si>
@@ -693,42 +909,63 @@
     <t>0,028 s</t>
   </si>
   <si>
+    <t>TC-095</t>
+  </si>
+  <si>
     <t>testPawnCaptureIncludesFromColumn</t>
   </si>
   <si>
     <t>Gyalog ütés (from oszlop megjelenik) → 'exf5'</t>
   </si>
   <si>
+    <t>TC-096</t>
+  </si>
+  <si>
     <t>testKnightMoveNotation</t>
   </si>
   <si>
     <t>Huszár lépés notáció → 'Nf3'</t>
   </si>
   <si>
+    <t>TC-097</t>
+  </si>
+  <si>
     <t>testBishopMoveNotation</t>
   </si>
   <si>
     <t>Futó lépés notáció → 'Be5'</t>
   </si>
   <si>
+    <t>TC-098</t>
+  </si>
+  <si>
     <t>testRookMoveNotation</t>
   </si>
   <si>
     <t>Bástya lépés notáció → 'Re1'</t>
   </si>
   <si>
+    <t>TC-099</t>
+  </si>
+  <si>
     <t>testQueenMoveNotation</t>
   </si>
   <si>
     <t>Vezér lépés notáció → 'Qd4'</t>
   </si>
   <si>
+    <t>TC-100</t>
+  </si>
+  <si>
     <t>testKingMoveNotation</t>
   </si>
   <si>
     <t>Király lépés notáció → 'Ke5'</t>
   </si>
   <si>
+    <t>TC-101</t>
+  </si>
+  <si>
     <t>testRookCaptureNotation</t>
   </si>
   <si>
@@ -775,6 +1012,18 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>TC-102</t>
+  </si>
+  <si>
+    <t>TC-103</t>
+  </si>
+  <si>
+    <t>TC-104</t>
+  </si>
+  <si>
+    <t>TC-105</t>
   </si>
   <si>
     <t>WebSocket</t>
@@ -916,7 +1165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -987,18 +1236,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1312,7 +1549,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>236</v>
+        <v>315</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
@@ -1341,13 +1578,13 @@
         <v>9</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>237</v>
+        <v>316</v>
       </c>
       <c r="G2" s="14">
         <v>46134</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>242</v>
+        <v>321</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>13</v>
@@ -1370,13 +1607,13 @@
         <v>9</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>237</v>
+        <v>316</v>
       </c>
       <c r="G3" s="13">
         <v>46134</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>241</v>
+        <v>320</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>13</v>
@@ -1399,13 +1636,13 @@
         <v>9</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>237</v>
+        <v>316</v>
       </c>
       <c r="G4" s="14">
         <v>46134</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>240</v>
+        <v>319</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>13</v>
@@ -1428,13 +1665,13 @@
         <v>9</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>237</v>
+        <v>316</v>
       </c>
       <c r="G5" s="13">
         <v>46134</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>239</v>
+        <v>318</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>13</v>
@@ -1448,22 +1685,22 @@
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>251</v>
+        <v>334</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>250</v>
+        <v>333</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G6" s="14">
         <v>46134</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>253</v>
+        <v>336</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>13</v>
@@ -1477,22 +1714,22 @@
         <v>9</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>252</v>
+        <v>335</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>250</v>
+        <v>333</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G7" s="13">
         <v>46134</v>
       </c>
       <c r="H7" s="25" t="s">
-        <v>254</v>
+        <v>337</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>13</v>
@@ -1515,7 +1752,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G8" s="14">
         <v>46134</v>
@@ -1544,7 +1781,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G9" s="13">
         <v>46134</v>
@@ -1573,7 +1810,7 @@
         <v>12</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G10" s="14">
         <v>46134</v>
@@ -1602,7 +1839,7 @@
         <v>12</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G11" s="13">
         <v>46134</v>
@@ -1631,7 +1868,7 @@
         <v>12</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G12" s="14">
         <v>46134</v>
@@ -1660,7 +1897,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G13" s="13">
         <v>46134</v>
@@ -1689,7 +1926,7 @@
         <v>12</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G14" s="14">
         <v>46134</v>
@@ -1718,7 +1955,7 @@
         <v>12</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G15" s="13">
         <v>46134</v>
@@ -1747,7 +1984,7 @@
         <v>12</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G16" s="14">
         <v>46134</v>
@@ -1776,7 +2013,7 @@
         <v>12</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G17" s="13">
         <v>46134</v>
@@ -1805,7 +2042,7 @@
         <v>12</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G18" s="14">
         <v>46134</v>
@@ -1834,7 +2071,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G19" s="13">
         <v>46134</v>
@@ -1863,7 +2100,7 @@
         <v>12</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G20" s="14">
         <v>46134</v>
@@ -1892,7 +2129,7 @@
         <v>12</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G21" s="13">
         <v>46134</v>
@@ -1921,7 +2158,7 @@
         <v>12</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G22" s="14">
         <v>46134</v>
@@ -1950,7 +2187,7 @@
         <v>12</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G23" s="13">
         <v>46134</v>
@@ -1979,7 +2216,7 @@
         <v>12</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G24" s="14">
         <v>46134</v>
@@ -2008,7 +2245,7 @@
         <v>12</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G25" s="13">
         <v>46134</v>
@@ -2037,7 +2274,7 @@
         <v>12</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G26" s="14">
         <v>46134</v>
@@ -2066,7 +2303,7 @@
         <v>12</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G27" s="13">
         <v>46134</v>
@@ -2095,7 +2332,7 @@
         <v>12</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G28" s="14">
         <v>46134</v>
@@ -2124,7 +2361,7 @@
         <v>12</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G29" s="13">
         <v>46134</v>
@@ -2153,7 +2390,7 @@
         <v>12</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G30" s="14">
         <v>46134</v>
@@ -2182,7 +2419,7 @@
         <v>12</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G31" s="13">
         <v>46134</v>
@@ -2211,7 +2448,7 @@
         <v>12</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G32" s="14">
         <v>46134</v>
@@ -2240,7 +2477,7 @@
         <v>12</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G33" s="13">
         <v>46134</v>
@@ -2269,7 +2506,7 @@
         <v>12</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G34" s="14">
         <v>46134</v>
@@ -2298,7 +2535,7 @@
         <v>12</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G35" s="13">
         <v>46134</v>
@@ -2327,7 +2564,7 @@
         <v>12</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G36" s="14">
         <v>46134</v>
@@ -2356,7 +2593,7 @@
         <v>12</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G37" s="13">
         <v>46134</v>
@@ -2385,7 +2622,7 @@
         <v>12</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G38" s="14">
         <v>46134</v>
@@ -2399,7 +2636,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>111</v>
@@ -2414,7 +2651,7 @@
         <v>12</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G39" s="13">
         <v>46134</v>
@@ -2428,13 +2665,13 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>130</v>
+        <v>163</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>131</v>
+        <v>164</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>23</v>
@@ -2443,13 +2680,13 @@
         <v>12</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G40" s="14">
         <v>46134</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>13</v>
@@ -2457,13 +2694,13 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>134</v>
+        <v>167</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>23</v>
@@ -2472,13 +2709,13 @@
         <v>12</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G41" s="13">
         <v>46134</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="I41" s="5" t="s">
         <v>13</v>
@@ -2486,13 +2723,13 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>137</v>
+        <v>170</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>23</v>
@@ -2501,13 +2738,13 @@
         <v>12</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G42" s="14">
         <v>46134</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>13</v>
@@ -2515,13 +2752,13 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>140</v>
+        <v>173</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>141</v>
+        <v>174</v>
       </c>
       <c r="D43" s="9" t="s">
         <v>23</v>
@@ -2530,13 +2767,13 @@
         <v>12</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G43" s="13">
         <v>46134</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>13</v>
@@ -2544,13 +2781,13 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>143</v>
+        <v>176</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>144</v>
+        <v>177</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>23</v>
@@ -2559,13 +2796,13 @@
         <v>12</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G44" s="14">
         <v>46134</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>13</v>
@@ -2573,13 +2810,13 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>148</v>
+        <v>185</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>149</v>
+        <v>186</v>
       </c>
       <c r="D45" s="9" t="s">
         <v>23</v>
@@ -2588,13 +2825,13 @@
         <v>12</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G45" s="13">
         <v>46134</v>
       </c>
       <c r="H45" s="9" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>13</v>
@@ -2602,13 +2839,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>152</v>
+        <v>189</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>153</v>
+        <v>190</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>23</v>
@@ -2617,13 +2854,13 @@
         <v>12</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G46" s="14">
         <v>46134</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
       <c r="I46" s="5" t="s">
         <v>13</v>
@@ -2631,13 +2868,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>155</v>
+        <v>192</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>156</v>
+        <v>193</v>
       </c>
       <c r="D47" s="9" t="s">
         <v>23</v>
@@ -2646,13 +2883,13 @@
         <v>12</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G47" s="13">
         <v>46134</v>
       </c>
       <c r="H47" s="9" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>13</v>
@@ -2660,13 +2897,13 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>158</v>
+        <v>195</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>159</v>
+        <v>196</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>23</v>
@@ -2675,13 +2912,13 @@
         <v>12</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G48" s="14">
         <v>46134</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
       <c r="I48" s="5" t="s">
         <v>13</v>
@@ -2689,13 +2926,13 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>161</v>
+        <v>198</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>162</v>
+        <v>199</v>
       </c>
       <c r="D49" s="9" t="s">
         <v>23</v>
@@ -2704,13 +2941,13 @@
         <v>12</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G49" s="13">
         <v>46134</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
       <c r="I49" s="5" t="s">
         <v>13</v>
@@ -2718,13 +2955,13 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>164</v>
+        <v>201</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>165</v>
+        <v>202</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>23</v>
@@ -2733,13 +2970,13 @@
         <v>12</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G50" s="14">
         <v>46134</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I50" s="5" t="s">
         <v>13</v>
@@ -2747,13 +2984,13 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>168</v>
+        <v>205</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>169</v>
+        <v>206</v>
       </c>
       <c r="D51" s="9" t="s">
         <v>23</v>
@@ -2762,13 +2999,13 @@
         <v>12</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G51" s="13">
         <v>46134</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I51" s="5" t="s">
         <v>13</v>
@@ -2776,13 +3013,13 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>127</v>
+        <v>156</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>171</v>
+        <v>208</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>172</v>
+        <v>209</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>23</v>
@@ -2791,13 +3028,13 @@
         <v>12</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G52" s="14">
         <v>46134</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I52" s="5" t="s">
         <v>13</v>
@@ -2805,13 +3042,13 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>128</v>
+        <v>159</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>174</v>
+        <v>211</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>175</v>
+        <v>212</v>
       </c>
       <c r="D53" s="9" t="s">
         <v>23</v>
@@ -2820,13 +3057,13 @@
         <v>12</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G53" s="13">
         <v>46134</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I53" s="5" t="s">
         <v>13</v>
@@ -2834,13 +3071,13 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>129</v>
+        <v>162</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>177</v>
+        <v>214</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>178</v>
+        <v>215</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>23</v>
@@ -2849,13 +3086,13 @@
         <v>12</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G54" s="14">
         <v>46134</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I54" s="5" t="s">
         <v>13</v>
@@ -2863,13 +3100,13 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>133</v>
+        <v>166</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>180</v>
+        <v>217</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>181</v>
+        <v>218</v>
       </c>
       <c r="D55" s="9" t="s">
         <v>23</v>
@@ -2878,13 +3115,13 @@
         <v>12</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G55" s="13">
         <v>46134</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I55" s="5" t="s">
         <v>13</v>
@@ -2892,13 +3129,13 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>136</v>
+        <v>169</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>183</v>
+        <v>220</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>184</v>
+        <v>221</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>23</v>
@@ -2907,13 +3144,13 @@
         <v>12</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G56" s="14">
         <v>46134</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I56" s="5" t="s">
         <v>13</v>
@@ -2921,13 +3158,13 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>139</v>
+        <v>172</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>186</v>
+        <v>223</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>187</v>
+        <v>224</v>
       </c>
       <c r="D57" s="9" t="s">
         <v>23</v>
@@ -2936,13 +3173,13 @@
         <v>12</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G57" s="13">
         <v>46134</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I57" s="5" t="s">
         <v>13</v>
@@ -2950,13 +3187,13 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>142</v>
+        <v>175</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>189</v>
+        <v>226</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>190</v>
+        <v>227</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>23</v>
@@ -2965,13 +3202,13 @@
         <v>12</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G58" s="14">
         <v>46134</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I58" s="5" t="s">
         <v>13</v>
@@ -2979,13 +3216,13 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>145</v>
+        <v>178</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>192</v>
+        <v>229</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>193</v>
+        <v>230</v>
       </c>
       <c r="D59" s="9" t="s">
         <v>23</v>
@@ -2994,13 +3231,13 @@
         <v>12</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G59" s="13">
         <v>46134</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I59" s="5" t="s">
         <v>13</v>
@@ -3008,13 +3245,13 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>146</v>
+        <v>181</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>195</v>
+        <v>232</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>196</v>
+        <v>233</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>23</v>
@@ -3023,13 +3260,13 @@
         <v>12</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G60" s="14">
         <v>46134</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I60" s="5" t="s">
         <v>13</v>
@@ -3037,13 +3274,13 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>147</v>
+        <v>184</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>198</v>
+        <v>235</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>199</v>
+        <v>236</v>
       </c>
       <c r="D61" s="9" t="s">
         <v>23</v>
@@ -3052,13 +3289,13 @@
         <v>12</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G61" s="13">
         <v>46134</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I61" s="5" t="s">
         <v>13</v>
@@ -3066,13 +3303,13 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>151</v>
+        <v>188</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>201</v>
+        <v>238</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>202</v>
+        <v>239</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>23</v>
@@ -3081,13 +3318,13 @@
         <v>12</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G62" s="14">
         <v>46134</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>166</v>
+        <v>203</v>
       </c>
       <c r="I62" s="5" t="s">
         <v>13</v>
@@ -3095,13 +3332,13 @@
     </row>
     <row r="63" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>154</v>
+        <v>191</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>204</v>
+        <v>241</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>205</v>
+        <v>242</v>
       </c>
       <c r="D63" s="9" t="s">
         <v>23</v>
@@ -3110,13 +3347,13 @@
         <v>12</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G63" s="13">
         <v>46134</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
       <c r="I63" s="5" t="s">
         <v>13</v>
@@ -3124,13 +3361,13 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>157</v>
+        <v>194</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>207</v>
+        <v>245</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>208</v>
+        <v>246</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>23</v>
@@ -3139,13 +3376,13 @@
         <v>12</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G64" s="14">
         <v>46134</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
       <c r="I64" s="5" t="s">
         <v>13</v>
@@ -3153,13 +3390,13 @@
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>160</v>
+        <v>197</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>209</v>
+        <v>248</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>210</v>
+        <v>249</v>
       </c>
       <c r="D65" s="9" t="s">
         <v>23</v>
@@ -3168,13 +3405,13 @@
         <v>12</v>
       </c>
       <c r="F65" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G65" s="13">
         <v>46134</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
       <c r="I65" s="5" t="s">
         <v>13</v>
@@ -3182,13 +3419,13 @@
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>163</v>
+        <v>200</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>211</v>
+        <v>251</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>212</v>
+        <v>252</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>23</v>
@@ -3197,13 +3434,13 @@
         <v>12</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G66" s="14">
         <v>46134</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
       <c r="I66" s="5" t="s">
         <v>13</v>
@@ -3211,13 +3448,13 @@
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>167</v>
+        <v>204</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>213</v>
+        <v>254</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>214</v>
+        <v>255</v>
       </c>
       <c r="D67" s="9" t="s">
         <v>23</v>
@@ -3226,13 +3463,13 @@
         <v>12</v>
       </c>
       <c r="F67" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G67" s="13">
         <v>46134</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
       <c r="I67" s="5" t="s">
         <v>13</v>
@@ -3240,13 +3477,13 @@
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>170</v>
+        <v>207</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>215</v>
+        <v>257</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>216</v>
+        <v>258</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>23</v>
@@ -3255,13 +3492,13 @@
         <v>12</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G68" s="14">
         <v>46134</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
       <c r="I68" s="5" t="s">
         <v>13</v>
@@ -3269,13 +3506,13 @@
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>173</v>
+        <v>210</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>217</v>
+        <v>260</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>218</v>
+        <v>261</v>
       </c>
       <c r="D69" s="9" t="s">
         <v>23</v>
@@ -3284,13 +3521,13 @@
         <v>12</v>
       </c>
       <c r="F69" s="9" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G69" s="13">
         <v>46134</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
       <c r="I69" s="5" t="s">
         <v>13</v>
@@ -3298,13 +3535,13 @@
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>176</v>
+        <v>213</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>219</v>
+        <v>291</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>220</v>
+        <v>292</v>
       </c>
       <c r="D70" s="12" t="s">
         <v>23</v>
@@ -3313,13 +3550,13 @@
         <v>12</v>
       </c>
       <c r="F70" s="12" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G70" s="15">
         <v>46134</v>
       </c>
       <c r="H70" s="12" t="s">
-        <v>221</v>
+        <v>293</v>
       </c>
       <c r="I70" s="5" t="s">
         <v>13</v>
@@ -3327,13 +3564,13 @@
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
-        <v>179</v>
+        <v>216</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>222</v>
+        <v>295</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>223</v>
+        <v>296</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>23</v>
@@ -3342,13 +3579,13 @@
         <v>12</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G71" s="16">
         <v>46134</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>221</v>
+        <v>293</v>
       </c>
       <c r="I71" s="5" t="s">
         <v>13</v>
@@ -3356,13 +3593,13 @@
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>182</v>
+        <v>219</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>224</v>
+        <v>298</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>225</v>
+        <v>299</v>
       </c>
       <c r="D72" s="12" t="s">
         <v>23</v>
@@ -3371,13 +3608,13 @@
         <v>12</v>
       </c>
       <c r="F72" s="12" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G72" s="15">
         <v>46134</v>
       </c>
       <c r="H72" s="12" t="s">
-        <v>221</v>
+        <v>293</v>
       </c>
       <c r="I72" s="5" t="s">
         <v>13</v>
@@ -3385,13 +3622,13 @@
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
-        <v>185</v>
+        <v>222</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>226</v>
+        <v>301</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>227</v>
+        <v>302</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>23</v>
@@ -3400,13 +3637,13 @@
         <v>12</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G73" s="16">
         <v>46134</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>221</v>
+        <v>293</v>
       </c>
       <c r="I73" s="5" t="s">
         <v>13</v>
@@ -3414,13 +3651,13 @@
     </row>
     <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>188</v>
+        <v>225</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>228</v>
+        <v>304</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>229</v>
+        <v>305</v>
       </c>
       <c r="D74" s="12" t="s">
         <v>23</v>
@@ -3429,13 +3666,13 @@
         <v>12</v>
       </c>
       <c r="F74" s="12" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G74" s="15">
         <v>46134</v>
       </c>
       <c r="H74" s="12" t="s">
-        <v>221</v>
+        <v>293</v>
       </c>
       <c r="I74" s="5" t="s">
         <v>13</v>
@@ -3443,13 +3680,13 @@
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
-        <v>191</v>
+        <v>228</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>230</v>
+        <v>307</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>231</v>
+        <v>308</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>23</v>
@@ -3458,13 +3695,13 @@
         <v>12</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G75" s="16">
         <v>46134</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>221</v>
+        <v>293</v>
       </c>
       <c r="I75" s="5" t="s">
         <v>13</v>
@@ -3472,13 +3709,13 @@
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>194</v>
+        <v>231</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>232</v>
+        <v>310</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>233</v>
+        <v>311</v>
       </c>
       <c r="D76" s="12" t="s">
         <v>23</v>
@@ -3487,13 +3724,13 @@
         <v>12</v>
       </c>
       <c r="F76" s="12" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G76" s="15">
         <v>46134</v>
       </c>
       <c r="H76" s="12" t="s">
-        <v>221</v>
+        <v>293</v>
       </c>
       <c r="I76" s="5" t="s">
         <v>13</v>
@@ -3501,13 +3738,13 @@
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>197</v>
+        <v>234</v>
       </c>
       <c r="B77" s="22" t="s">
-        <v>243</v>
+        <v>322</v>
       </c>
       <c r="C77" s="22" t="s">
-        <v>245</v>
+        <v>324</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>23</v>
@@ -3516,30 +3753,30 @@
         <v>12</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G77" s="16">
         <v>46135</v>
       </c>
       <c r="H77" s="19" t="s">
-        <v>247</v>
+        <v>326</v>
       </c>
       <c r="I77" s="5" t="s">
         <v>13</v>
       </c>
       <c r="K77" t="s">
-        <v>249</v>
+        <v>328</v>
       </c>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>200</v>
+        <v>237</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>244</v>
+        <v>323</v>
       </c>
       <c r="C78" s="23" t="s">
-        <v>246</v>
+        <v>325</v>
       </c>
       <c r="D78" s="12" t="s">
         <v>23</v>
@@ -3548,13 +3785,13 @@
         <v>12</v>
       </c>
       <c r="F78" s="12" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G78" s="15">
         <v>46136</v>
       </c>
       <c r="H78" s="21" t="s">
-        <v>248</v>
+        <v>327</v>
       </c>
       <c r="I78" s="5" t="s">
         <v>13</v>
@@ -3562,13 +3799,13 @@
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
-        <v>203</v>
+        <v>240</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>234</v>
+        <v>313</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>235</v>
+        <v>314</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>23</v>
@@ -3577,13 +3814,13 @@
         <v>12</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>238</v>
+        <v>317</v>
       </c>
       <c r="G79" s="16">
         <v>46134</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>221</v>
+        <v>293</v>
       </c>
       <c r="I79" s="5" t="s">
         <v>13</v>
@@ -3591,305 +3828,791 @@
       <c r="J79" s="20"/>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A80" s="26"/>
-      <c r="B80" s="27"/>
-      <c r="C80" s="27"/>
-      <c r="D80" s="26"/>
-      <c r="E80" s="26"/>
-      <c r="F80" s="26"/>
-      <c r="G80" s="28"/>
-      <c r="H80" s="26"/>
-      <c r="I80" s="29"/>
+      <c r="A80" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="C80" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="D80" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E80" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G80" s="15">
+        <v>46134</v>
+      </c>
+      <c r="H80" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="I80" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="P80" s="17"/>
       <c r="Q80" s="17"/>
     </row>
     <row r="81" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A81" s="26"/>
-      <c r="B81" s="27"/>
-      <c r="C81" s="27"/>
-      <c r="D81" s="26"/>
-      <c r="E81" s="26"/>
-      <c r="F81" s="26"/>
-      <c r="G81" s="28"/>
-      <c r="H81" s="26"/>
-      <c r="I81" s="29"/>
+      <c r="A81" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="B81" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C81" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F81" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G81" s="16">
+        <v>46134</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="I81" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="P81" s="17"/>
       <c r="Q81" s="17"/>
     </row>
     <row r="82" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A82" s="26"/>
-      <c r="B82" s="27"/>
-      <c r="C82" s="27"/>
-      <c r="D82" s="26"/>
-      <c r="E82" s="26"/>
-      <c r="F82" s="26"/>
-      <c r="G82" s="28"/>
-      <c r="H82" s="26"/>
-      <c r="I82" s="29"/>
+      <c r="A82" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G82" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I82" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="83" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A83" s="26"/>
-      <c r="B83" s="27"/>
-      <c r="C83" s="27"/>
-      <c r="D83" s="26"/>
-      <c r="E83" s="26"/>
-      <c r="F83" s="26"/>
-      <c r="G83" s="28"/>
-      <c r="H83" s="26"/>
-      <c r="I83" s="29"/>
+      <c r="A83" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C83" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E83" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F83" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G83" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H83" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I83" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A84" s="26"/>
-      <c r="B84" s="27"/>
-      <c r="C84" s="27"/>
-      <c r="D84" s="26"/>
-      <c r="E84" s="26"/>
-      <c r="F84" s="26"/>
-      <c r="G84" s="28"/>
-      <c r="H84" s="26"/>
-      <c r="I84" s="29"/>
+      <c r="A84" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G84" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I84" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="85" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A85" s="26"/>
-      <c r="B85" s="27"/>
-      <c r="C85" s="27"/>
-      <c r="D85" s="26"/>
-      <c r="E85" s="26"/>
-      <c r="F85" s="26"/>
-      <c r="G85" s="28"/>
-      <c r="H85" s="26"/>
-      <c r="I85" s="29"/>
+      <c r="A85" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="B85" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D85" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E85" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F85" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G85" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H85" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I85" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A86" s="26"/>
-      <c r="B86" s="27"/>
-      <c r="C86" s="27"/>
-      <c r="D86" s="26"/>
-      <c r="E86" s="26"/>
-      <c r="F86" s="26"/>
-      <c r="G86" s="28"/>
-      <c r="H86" s="26"/>
-      <c r="I86" s="29"/>
+      <c r="A86" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G86" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I86" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="87" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A87" s="26"/>
-      <c r="B87" s="27"/>
-      <c r="C87" s="27"/>
-      <c r="D87" s="26"/>
-      <c r="E87" s="26"/>
-      <c r="F87" s="26"/>
-      <c r="G87" s="28"/>
-      <c r="H87" s="26"/>
-      <c r="I87" s="29"/>
+      <c r="A87" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="B87" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E87" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G87" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H87" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I87" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A88" s="26"/>
-      <c r="B88" s="27"/>
-      <c r="C88" s="27"/>
-      <c r="D88" s="26"/>
-      <c r="E88" s="26"/>
-      <c r="F88" s="26"/>
-      <c r="G88" s="28"/>
-      <c r="H88" s="26"/>
-      <c r="I88" s="29"/>
+      <c r="A88" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G88" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I88" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A89" s="26"/>
-      <c r="B89" s="27"/>
-      <c r="C89" s="27"/>
-      <c r="D89" s="26"/>
-      <c r="E89" s="26"/>
-      <c r="F89" s="26"/>
-      <c r="G89" s="28"/>
-      <c r="H89" s="26"/>
-      <c r="I89" s="29"/>
+      <c r="A89" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="B89" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C89" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D89" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E89" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F89" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G89" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H89" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I89" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A90" s="26"/>
-      <c r="B90" s="27"/>
-      <c r="C90" s="27"/>
-      <c r="D90" s="26"/>
-      <c r="E90" s="26"/>
-      <c r="F90" s="26"/>
-      <c r="G90" s="28"/>
-      <c r="H90" s="26"/>
-      <c r="I90" s="29"/>
+      <c r="A90" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G90" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I90" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A91" s="26"/>
-      <c r="B91" s="27"/>
-      <c r="C91" s="27"/>
-      <c r="D91" s="26"/>
-      <c r="E91" s="26"/>
-      <c r="F91" s="26"/>
-      <c r="G91" s="28"/>
-      <c r="H91" s="26"/>
-      <c r="I91" s="29"/>
+      <c r="A91" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="B91" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="D91" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E91" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F91" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G91" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H91" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I91" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="92" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A92" s="26"/>
-      <c r="B92" s="27"/>
-      <c r="C92" s="27"/>
-      <c r="D92" s="26"/>
-      <c r="E92" s="26"/>
-      <c r="F92" s="26"/>
-      <c r="G92" s="28"/>
-      <c r="H92" s="26"/>
-      <c r="I92" s="29"/>
+      <c r="A92" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G92" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I92" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="93" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A93" s="26"/>
-      <c r="B93" s="27"/>
-      <c r="C93" s="27"/>
-      <c r="D93" s="26"/>
-      <c r="E93" s="26"/>
-      <c r="F93" s="26"/>
-      <c r="G93" s="28"/>
-      <c r="H93" s="26"/>
-      <c r="I93" s="29"/>
+      <c r="A93" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="B93" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C93" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D93" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E93" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F93" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G93" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H93" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I93" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="94" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A94" s="26"/>
-      <c r="B94" s="27"/>
-      <c r="C94" s="27"/>
-      <c r="D94" s="26"/>
-      <c r="E94" s="26"/>
-      <c r="F94" s="26"/>
-      <c r="G94" s="28"/>
-      <c r="H94" s="26"/>
-      <c r="I94" s="29"/>
+      <c r="A94" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G94" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I94" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="95" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A95" s="26"/>
-      <c r="B95" s="27"/>
-      <c r="C95" s="27"/>
-      <c r="D95" s="26"/>
-      <c r="E95" s="26"/>
-      <c r="F95" s="26"/>
-      <c r="G95" s="28"/>
-      <c r="H95" s="26"/>
-      <c r="I95" s="29"/>
+      <c r="A95" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="B95" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C95" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="D95" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E95" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F95" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G95" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H95" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I95" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="96" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A96" s="26"/>
-      <c r="B96" s="27"/>
-      <c r="C96" s="27"/>
-      <c r="D96" s="26"/>
-      <c r="E96" s="26"/>
-      <c r="F96" s="26"/>
-      <c r="G96" s="28"/>
-      <c r="H96" s="26"/>
-      <c r="I96" s="29"/>
+      <c r="A96" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B96" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="C96" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="D96" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E96" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F96" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="G96" s="15">
+        <v>46134</v>
+      </c>
+      <c r="H96" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="I96" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A97" s="26"/>
-      <c r="B97" s="27"/>
-      <c r="C97" s="27"/>
-      <c r="D97" s="26"/>
-      <c r="E97" s="26"/>
-      <c r="F97" s="26"/>
-      <c r="G97" s="28"/>
-      <c r="H97" s="26"/>
-      <c r="I97" s="29"/>
+      <c r="A97" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="B97" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="C97" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F97" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="G97" s="16">
+        <v>46134</v>
+      </c>
+      <c r="H97" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="I97" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A98" s="26"/>
-      <c r="B98" s="27"/>
-      <c r="C98" s="27"/>
-      <c r="D98" s="26"/>
-      <c r="E98" s="26"/>
-      <c r="F98" s="26"/>
-      <c r="G98" s="28"/>
-      <c r="H98" s="26"/>
-      <c r="I98" s="29"/>
+      <c r="A98" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B98" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="C98" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D98" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E98" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G98" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H98" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="I98" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" s="26"/>
-      <c r="B99" s="27"/>
-      <c r="C99" s="27"/>
-      <c r="D99" s="26"/>
-      <c r="E99" s="26"/>
-      <c r="F99" s="26"/>
-      <c r="G99" s="28"/>
-      <c r="H99" s="26"/>
-      <c r="I99" s="29"/>
+      <c r="A99" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="B99" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="C99" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="D99" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F99" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G99" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H99" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="I99" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" s="26"/>
-      <c r="B100" s="27"/>
-      <c r="C100" s="27"/>
-      <c r="D100" s="26"/>
-      <c r="E100" s="26"/>
-      <c r="F100" s="26"/>
-      <c r="G100" s="28"/>
-      <c r="H100" s="26"/>
-      <c r="I100" s="29"/>
+      <c r="A100" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B100" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="C100" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="D100" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E100" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G100" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H100" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="I100" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A101" s="26"/>
-      <c r="B101" s="27"/>
-      <c r="C101" s="27"/>
-      <c r="D101" s="26"/>
-      <c r="E101" s="26"/>
-      <c r="F101" s="26"/>
-      <c r="G101" s="28"/>
-      <c r="H101" s="26"/>
-      <c r="I101" s="29"/>
+      <c r="A101" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="B101" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="C101" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="D101" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F101" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G101" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H101" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="I101" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A102" s="26"/>
-      <c r="B102" s="27"/>
-      <c r="C102" s="27"/>
-      <c r="D102" s="26"/>
-      <c r="E102" s="26"/>
-      <c r="F102" s="26"/>
-      <c r="G102" s="28"/>
-      <c r="H102" s="26"/>
-      <c r="I102" s="29"/>
+      <c r="A102" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B102" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="C102" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="D102" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E102" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G102" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H102" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="I102" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A103" s="26"/>
-      <c r="B103" s="27"/>
-      <c r="C103" s="27"/>
-      <c r="D103" s="26"/>
-      <c r="E103" s="26"/>
-      <c r="F103" s="26"/>
-      <c r="G103" s="28"/>
-      <c r="H103" s="26"/>
-      <c r="I103" s="29"/>
+      <c r="A103" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="B103" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="C103" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="D103" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F103" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G103" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H103" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="I103" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A104" s="26"/>
-      <c r="B104" s="27"/>
-      <c r="C104" s="27"/>
-      <c r="D104" s="26"/>
-      <c r="E104" s="26"/>
-      <c r="F104" s="26"/>
-      <c r="G104" s="28"/>
-      <c r="H104" s="26"/>
-      <c r="I104" s="29"/>
+      <c r="A104" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B104" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="C104" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="D104" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E104" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G104" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H104" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="I104" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A105" s="26"/>
-      <c r="B105" s="27"/>
-      <c r="C105" s="27"/>
-      <c r="D105" s="26"/>
-      <c r="E105" s="26"/>
-      <c r="F105" s="26"/>
-      <c r="G105" s="28"/>
-      <c r="H105" s="26"/>
-      <c r="I105" s="29"/>
+      <c r="A105" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="B105" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="C105" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="D105" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E105" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F105" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="G105" s="13">
+        <v>46134</v>
+      </c>
+      <c r="H105" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="I105" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A106" s="26"/>
-      <c r="B106" s="27"/>
-      <c r="C106" s="27"/>
-      <c r="D106" s="26"/>
-      <c r="E106" s="26"/>
-      <c r="F106" s="26"/>
-      <c r="G106" s="28"/>
-      <c r="H106" s="26"/>
-      <c r="I106" s="29"/>
+      <c r="A106" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B106" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="C106" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="D106" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E106" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G106" s="14">
+        <v>46134</v>
+      </c>
+      <c r="H106" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="I106" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="113" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G113" s="18"/>

</xml_diff>